<commit_message>
Change Cases - add new testcase
</commit_message>
<xml_diff>
--- a/docs/Cases.xlsx
+++ b/docs/Cases.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="sRwcLHFO/e2p7cfFFBUEUHbIbm61vZrCZyYcbfcMveg="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="7Xk8VqOlAGMTVUzLAvd8aM4sgKzJx6ssyR1lHjStdak="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="325">
   <si>
     <t>ID</t>
   </si>
@@ -1048,6 +1048,66 @@
   </si>
   <si>
     <t>1. Порядок новостей идет от новых к старым</t>
+  </si>
+  <si>
+    <t>TC044</t>
+  </si>
+  <si>
+    <t>Редактирование существующей новости</t>
+  </si>
+  <si>
+    <t>Пользователь авторизован. На главной странице открыта панель управления новостями (Control Panel). Существует хотя бы одна созданная новость.</t>
+  </si>
+  <si>
+    <t>1. Создать новость с заголовком "Старый заголовок", категорией "Объявление" и описанием "Старое описание"</t>
+  </si>
+  <si>
+    <t>1. Новость успешно создана</t>
+  </si>
+  <si>
+    <t>2. Нажать на кнопку сортировки для обновления списка</t>
+  </si>
+  <si>
+    <t>2. Список новостей отсортирован</t>
+  </si>
+  <si>
+    <t>3. Нажать на иконку редактирования (карандаш) у созданной новости</t>
+  </si>
+  <si>
+    <t>3. Открывается страница редактирования новости</t>
+  </si>
+  <si>
+    <t>4. В поле "Title" ввести новый заголовок "Новый заголовок"</t>
+  </si>
+  <si>
+    <t>5. В поле "Description" ввести новое описание "Обновлённое описание"</t>
+  </si>
+  <si>
+    <t>6. Новость сохранена, происходит возврат на страницу панели управления</t>
+  </si>
+  <si>
+    <t>7. Проверить, что старый заголовок отсутствует в списке</t>
+  </si>
+  <si>
+    <t>7. Старый заголовок не отображается</t>
+  </si>
+  <si>
+    <t>8. Проверить, что новый заголовок отображается в списке</t>
+  </si>
+  <si>
+    <t>8. Новый заголовок виден</t>
+  </si>
+  <si>
+    <t>9. Нажать на заголовок новой новости для раскрытия карточки</t>
+  </si>
+  <si>
+    <t>9. Карточка раскрывается</t>
+  </si>
+  <si>
+    <t>10. Проверить, что новое описание отображается</t>
+  </si>
+  <si>
+    <t>10. Новое описание видно</t>
   </si>
 </sst>
 </file>
@@ -4600,8 +4660,160 @@
         <v>1</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B186" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C186" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D186" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E186" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="F186" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="G186" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="H186" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="13"/>
+      <c r="B187" s="13"/>
+      <c r="C187" s="13"/>
+      <c r="D187" s="13"/>
+      <c r="E187" s="13"/>
+      <c r="F187" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="G187" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="H187" s="13"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="13"/>
+      <c r="B188" s="13"/>
+      <c r="C188" s="13"/>
+      <c r="D188" s="13"/>
+      <c r="E188" s="13"/>
+      <c r="F188" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="G188" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="H188" s="13"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="13"/>
+      <c r="B189" s="13"/>
+      <c r="C189" s="13"/>
+      <c r="D189" s="13"/>
+      <c r="E189" s="13"/>
+      <c r="F189" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="G189" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="H189" s="13"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="13"/>
+      <c r="B190" s="13"/>
+      <c r="C190" s="13"/>
+      <c r="D190" s="13"/>
+      <c r="E190" s="13"/>
+      <c r="F190" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="G190" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="H190" s="13"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="13"/>
+      <c r="B191" s="13"/>
+      <c r="C191" s="13"/>
+      <c r="D191" s="13"/>
+      <c r="E191" s="13"/>
+      <c r="F191" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="G191" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="H191" s="13"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="13"/>
+      <c r="B192" s="13"/>
+      <c r="C192" s="13"/>
+      <c r="D192" s="13"/>
+      <c r="E192" s="13"/>
+      <c r="F192" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="G192" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="H192" s="13"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="13"/>
+      <c r="B193" s="13"/>
+      <c r="C193" s="13"/>
+      <c r="D193" s="13"/>
+      <c r="E193" s="13"/>
+      <c r="F193" s="11" t="s">
+        <v>319</v>
+      </c>
+      <c r="G193" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="H193" s="13"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="13"/>
+      <c r="B194" s="13"/>
+      <c r="C194" s="13"/>
+      <c r="D194" s="13"/>
+      <c r="E194" s="13"/>
+      <c r="F194" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="G194" s="11" t="s">
+        <v>322</v>
+      </c>
+      <c r="H194" s="13"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="14"/>
+      <c r="B195" s="14"/>
+      <c r="C195" s="14"/>
+      <c r="D195" s="14"/>
+      <c r="E195" s="14"/>
+      <c r="F195" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="G195" s="11" t="s">
+        <v>324</v>
+      </c>
+      <c r="H195" s="14"/>
+    </row>
   </sheetData>
-  <mergeCells count="227">
+  <mergeCells count="233">
     <mergeCell ref="B56:B58"/>
     <mergeCell ref="C56:C58"/>
     <mergeCell ref="B59:B63"/>
@@ -4675,6 +4887,18 @@
     <mergeCell ref="D169:D176"/>
     <mergeCell ref="E169:E176"/>
     <mergeCell ref="H169:H176"/>
+    <mergeCell ref="D177:D184"/>
+    <mergeCell ref="A186:A195"/>
+    <mergeCell ref="B186:B195"/>
+    <mergeCell ref="A177:A184"/>
+    <mergeCell ref="B177:B184"/>
+    <mergeCell ref="C177:C184"/>
+    <mergeCell ref="E177:E184"/>
+    <mergeCell ref="H177:H184"/>
+    <mergeCell ref="E186:E195"/>
+    <mergeCell ref="H186:H195"/>
+    <mergeCell ref="C186:C195"/>
+    <mergeCell ref="D186:D195"/>
     <mergeCell ref="D29:D31"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="A24:A28"/>
@@ -4709,12 +4933,6 @@
     <mergeCell ref="H53:H55"/>
     <mergeCell ref="A56:A58"/>
     <mergeCell ref="H56:H58"/>
-    <mergeCell ref="A177:A184"/>
-    <mergeCell ref="B177:B184"/>
-    <mergeCell ref="C177:C184"/>
-    <mergeCell ref="D177:D184"/>
-    <mergeCell ref="E177:E184"/>
-    <mergeCell ref="H177:H184"/>
     <mergeCell ref="D5:D7"/>
     <mergeCell ref="E5:E7"/>
     <mergeCell ref="D8:D10"/>
@@ -4831,7 +5049,7 @@
     <mergeCell ref="H110:H112"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="D2 D5 D8 D11 D14 D16 D18 D22:D24 D29 D32 D42 D53 D56 D59 D64 D72 D80 D84 D89 D93 D95 D97 D99 D101 D103 D105:D107 D110 D113 D117 D121 D123 D131 D141 D148 D155 D163 D169 D177 D185">
+    <dataValidation type="list" allowBlank="1" sqref="D2 D5 D8 D11 D14 D16 D18 D22:D24 D29 D32 D42 D53 D56 D59 D64 D72 D80 D84 D89 D93 D95 D97 D99 D101 D103 D105:D107 D110 D113 D117 D121 D123 D131 D141 D148 D155 D163 D169 D177 D185:D186">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update Cases and allure-results.zip
</commit_message>
<xml_diff>
--- a/docs/Cases.xlsx
+++ b/docs/Cases.xlsx
@@ -201,7 +201,7 @@
     <t>TC009</t>
   </si>
   <si>
-    <t>Однократное нажатие системной кнопки "Назад" на главной странице Main сворачивает приложение</t>
+    <t>Однократное нажатие системной кнопки "Назад" на главной странице Main закрывает приложение</t>
   </si>
   <si>
     <t>Low</t>
@@ -210,7 +210,7 @@
     <t>Пользователь авторизован и находится на главной странице Main</t>
   </si>
   <si>
-    <t>1. Пользователь остается на страницу Main, приложение не закрывается</t>
+    <t>1. Приложение закрывается</t>
   </si>
   <si>
     <t>TC010</t>
@@ -4887,18 +4887,16 @@
     <mergeCell ref="D169:D176"/>
     <mergeCell ref="E169:E176"/>
     <mergeCell ref="H169:H176"/>
-    <mergeCell ref="D177:D184"/>
-    <mergeCell ref="A186:A195"/>
-    <mergeCell ref="B186:B195"/>
+    <mergeCell ref="D186:D195"/>
+    <mergeCell ref="E186:E195"/>
     <mergeCell ref="A177:A184"/>
     <mergeCell ref="B177:B184"/>
     <mergeCell ref="C177:C184"/>
+    <mergeCell ref="D177:D184"/>
     <mergeCell ref="E177:E184"/>
     <mergeCell ref="H177:H184"/>
-    <mergeCell ref="E186:E195"/>
+    <mergeCell ref="A186:A195"/>
     <mergeCell ref="H186:H195"/>
-    <mergeCell ref="C186:C195"/>
-    <mergeCell ref="D186:D195"/>
     <mergeCell ref="D29:D31"/>
     <mergeCell ref="E29:E31"/>
     <mergeCell ref="A24:A28"/>
@@ -4933,6 +4931,8 @@
     <mergeCell ref="H53:H55"/>
     <mergeCell ref="A56:A58"/>
     <mergeCell ref="H56:H58"/>
+    <mergeCell ref="B186:B195"/>
+    <mergeCell ref="C186:C195"/>
     <mergeCell ref="D5:D7"/>
     <mergeCell ref="E5:E7"/>
     <mergeCell ref="D8:D10"/>

</xml_diff>